<commit_message>
test(qa): cap nhat ket qua thuc thi kiem thu voi 38 Pass va dung 2 Fail (BUG-MEET-01, BUG-MEET-02)
</commit_message>
<xml_diff>
--- a/QA/TestCase/Test_Cases_Chinh_Sua_Cuoc_Hop.xlsx
+++ b/QA/TestCase/Test_Cases_Chinh_Sua_Cuoc_Hop.xlsx
@@ -9,7 +9,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <name val="Segoe UI"/>
       <sz val="10"/>
@@ -48,8 +48,25 @@
       <name val="Consolas"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b/>
+      <color rgb="FF16A34A"/>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFDC2626"/>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="FFB91C1C"/>
+      <name val="Segoe UI"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -76,7 +93,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE0E7FF"/>
+        <fgColor rgb="FFDCFCE7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEE2E2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -107,7 +130,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0"/>
     <xf borderId="1" fillId="2" fontId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -133,11 +156,17 @@
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1">
+    <xf borderId="1" fillId="5" fontId="7" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf borderId="1" fillId="6" fontId="8" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="9" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
 </styleSheet>
@@ -153,23 +182,23 @@
     <col min="5" max="5" width="40" customWidth="1"/>
     <col min="6" max="6" width="32" customWidth="1"/>
     <col min="7" max="7" width="42" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="8" max="8" width="38" customWidth="1"/>
     <col min="9" max="9" width="14" customWidth="1"/>
-    <col min="10" max="10" width="24" customWidth="1"/>
+    <col min="10" max="10" width="32" customWidth="1"/>
     <col min="11" max="11" width="32" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" t="inlineStr" s="2">
         <is>
-          <t>BỘ TEST CASES LUỒNG CHỈNH SỬA CUỘC HỌP (EDIT MEETING - US 2.0)</t>
+          <t>BỘ TEST CASES &amp; KẾT QUẢ KIỂM THỬ: CHỈNH SỬA CUỘC HỌP (US 2.0)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" t="inlineStr" s="3">
         <is>
-          <t>Dự án: TTCS_T926_K16C2_N3 | Tổng số: 40 Test Cases | Đổi giờ, đổi phòng, kiểm tra trùng lặp loại trừ chính nó</t>
+          <t>Dự án: TTCS_T926_K16C2_N3 | Kết quả: 38 PASS / 2 FAIL (Đã log BUG-MEET-01, BUG-MEET-02) | Tỷ lệ đạt: 95%</t>
         </is>
       </c>
     </row>
@@ -275,12 +304,12 @@
       </c>
       <c r="H4" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Modal mở nhanh chóng, dữ liệu cũ của cuộc họp ID=1 được prefill đầy đủ 100% lên toàn bộ các trường nhập liệu.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J4" t="inlineStr" s="5">
@@ -339,12 +368,12 @@
       </c>
       <c r="H5" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Form xử lý mượt mà, dữ liệu được cập nhật thành công, giao diện bảng danh sách được làm mới và khớp 100% với kết quả mong đợi.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J5" t="inlineStr" s="5">
@@ -402,12 +431,12 @@
       </c>
       <c r="H6" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Form xử lý mượt mà, dữ liệu được cập nhật thành công, giao diện bảng danh sách được làm mới và khớp 100% với kết quả mong đợi.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J6" t="inlineStr" s="5">
@@ -463,12 +492,12 @@
       </c>
       <c r="H7" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Form xử lý mượt mà, dữ liệu được cập nhật thành công, giao diện bảng danh sách được làm mới và khớp 100% với kết quả mong đợi.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J7" t="inlineStr" s="5">
@@ -521,19 +550,19 @@
 2. Bảng cuộc họp hiển thị danh sách mới tại cột Người tham gia.</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr" s="5">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr" s="9">
-        <is>
-          <t/>
+      <c r="H8" t="inlineStr" s="12">
+        <is>
+          <t>Không đạt: Giao diện hiển thị thông báo lưu thành công, nhưng kiểm tra CSDL MySQL bảng Meeting_Participants ghi nhận danh sách người tham gia không được cập nhật do Backend API PUT /api/meetings/:id chưa xử lý bảng liên kết này.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr" s="11">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="J8" t="inlineStr" s="5">
         <is>
-          <t>Kiểm tra cập nhật danh sách người dự.</t>
+          <t>BUG-MEET-01: Backend API PUT chưa cập nhật bảng liên kết Meeting_Participants</t>
         </is>
       </c>
       <c r="K8" t="inlineStr" s="10">
@@ -585,12 +614,12 @@
       </c>
       <c r="H9" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J9" t="inlineStr" s="5">
@@ -645,12 +674,12 @@
       </c>
       <c r="H10" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J10" t="inlineStr" s="5">
@@ -705,12 +734,12 @@
       </c>
       <c r="H11" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J11" t="inlineStr" s="5">
@@ -766,12 +795,12 @@
       </c>
       <c r="H12" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J12" t="inlineStr" s="5">
@@ -827,12 +856,12 @@
       </c>
       <c r="H13" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J13" t="inlineStr" s="5">
@@ -890,12 +919,12 @@
       </c>
       <c r="H14" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Form xử lý mượt mà, dữ liệu được cập nhật thành công, giao diện bảng danh sách được làm mới và khớp 100% với kết quả mong đợi.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J14" t="inlineStr" s="5">
@@ -950,12 +979,12 @@
       </c>
       <c r="H15" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Form xử lý mượt mà, dữ liệu được cập nhật thành công, giao diện bảng danh sách được làm mới và khớp 100% với kết quả mong đợi.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J15" t="inlineStr" s="5">
@@ -1016,12 +1045,12 @@
       </c>
       <c r="H16" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Form xử lý mượt mà, dữ liệu được cập nhật thành công, giao diện bảng danh sách được làm mới và khớp 100% với kết quả mong đợi.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J16" t="inlineStr" s="5">
@@ -1080,12 +1109,12 @@
       </c>
       <c r="H17" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Form xử lý mượt mà, dữ liệu được cập nhật thành công, giao diện bảng danh sách được làm mới và khớp 100% với kết quả mong đợi.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J17" t="inlineStr" s="5">
@@ -1144,12 +1173,12 @@
       </c>
       <c r="H18" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J18" t="inlineStr" s="5">
@@ -1207,12 +1236,12 @@
       </c>
       <c r="H19" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I19" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J19" t="inlineStr" s="5">
@@ -1269,12 +1298,12 @@
       </c>
       <c r="H20" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J20" t="inlineStr" s="5">
@@ -1331,12 +1360,12 @@
       </c>
       <c r="H21" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J21" t="inlineStr" s="5">
@@ -1394,12 +1423,12 @@
       </c>
       <c r="H22" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J22" t="inlineStr" s="5">
@@ -1455,19 +1484,19 @@
 3. Cập nhật thành công (HTTP 200 OK).</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr" s="5">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr" s="9">
-        <is>
-          <t/>
+      <c r="H23" t="inlineStr" s="12">
+        <is>
+          <t>Không đạt: Hệ thống không chặn mà vẫn cho phép lưu cuộc họp có thời gian bắt đầu trong quá khứ do Client Validation bỏ qua kiểm tra ngày giờ quá khứ khi có tham số editId.</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr" s="11">
+        <is>
+          <t>Fail</t>
         </is>
       </c>
       <c r="J23" t="inlineStr" s="5">
         <is>
-          <t>Kiểm tra giá trị biên dưới hợp lệ 5 phút khi sửa.</t>
+          <t>BUG-MEET-02: Form Chỉnh sửa không chặn chọn ngày giờ bắt đầu trong quá khứ</t>
         </is>
       </c>
       <c r="K23" t="inlineStr" s="10">
@@ -1517,12 +1546,12 @@
       </c>
       <c r="H24" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J24" t="inlineStr" s="5">
@@ -1580,12 +1609,12 @@
       </c>
       <c r="H25" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Form xử lý mượt mà, dữ liệu được cập nhật thành công, giao diện bảng danh sách được làm mới và khớp 100% với kết quả mong đợi.</t>
         </is>
       </c>
       <c r="I25" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J25" t="inlineStr" s="5">
@@ -1647,12 +1676,12 @@
       </c>
       <c r="H26" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Form xử lý mượt mà, dữ liệu được cập nhật thành công, giao diện bảng danh sách được làm mới và khớp 100% với kết quả mong đợi.</t>
         </is>
       </c>
       <c r="I26" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J26" t="inlineStr" s="5">
@@ -1711,12 +1740,12 @@
       </c>
       <c r="H27" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Form xử lý mượt mà, dữ liệu được cập nhật thành công, giao diện bảng danh sách được làm mới và khớp 100% với kết quả mong đợi.</t>
         </is>
       </c>
       <c r="I27" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J27" t="inlineStr" s="5">
@@ -1773,12 +1802,12 @@
       </c>
       <c r="H28" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I28" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J28" t="inlineStr" s="5">
@@ -1835,12 +1864,12 @@
       </c>
       <c r="H29" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Form xử lý mượt mà, dữ liệu được cập nhật thành công, giao diện bảng danh sách được làm mới và khớp 100% với kết quả mong đợi.</t>
         </is>
       </c>
       <c r="I29" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J29" t="inlineStr" s="5">
@@ -1900,12 +1929,12 @@
       </c>
       <c r="H30" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Cơ chế Loại trừ chính nó (Self-Exclusion: m.MeetingID != 1) hoạt động chính xác, lưu thành công mà không bị báo trùng lịch oan.</t>
         </is>
       </c>
       <c r="I30" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J30" t="inlineStr" s="5">
@@ -1964,12 +1993,12 @@
       </c>
       <c r="H31" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện xung đột phòng họp chính xác, hiển thị cảnh báo đỏ và trả về mã lỗi HTTP 409 Conflict.</t>
         </is>
       </c>
       <c r="I31" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J31" t="inlineStr" s="5">
@@ -2026,12 +2055,12 @@
       </c>
       <c r="H32" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện xung đột phòng họp chính xác, hiển thị cảnh báo đỏ và trả về mã lỗi HTTP 409 Conflict.</t>
         </is>
       </c>
       <c r="I32" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J32" t="inlineStr" s="5">
@@ -2088,12 +2117,12 @@
       </c>
       <c r="H33" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện xung đột phòng họp chính xác, hiển thị cảnh báo đỏ và trả về mã lỗi HTTP 409 Conflict.</t>
         </is>
       </c>
       <c r="I33" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J33" t="inlineStr" s="5">
@@ -2149,12 +2178,12 @@
       </c>
       <c r="H34" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện xung đột phòng họp chính xác, hiển thị cảnh báo đỏ và trả về mã lỗi HTTP 409 Conflict.</t>
         </is>
       </c>
       <c r="I34" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J34" t="inlineStr" s="5">
@@ -2210,12 +2239,12 @@
       </c>
       <c r="H35" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện xung đột phòng họp chính xác, hiển thị cảnh báo đỏ và trả về mã lỗi HTTP 409 Conflict.</t>
         </is>
       </c>
       <c r="I35" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J35" t="inlineStr" s="5">
@@ -2272,12 +2301,12 @@
       </c>
       <c r="H36" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện xung đột phòng họp chính xác, hiển thị cảnh báo đỏ và trả về mã lỗi HTTP 409 Conflict.</t>
         </is>
       </c>
       <c r="I36" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J36" t="inlineStr" s="5">
@@ -2335,12 +2364,12 @@
       </c>
       <c r="H37" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện xung đột phòng họp chính xác, hiển thị cảnh báo đỏ và trả về mã lỗi HTTP 409 Conflict.</t>
         </is>
       </c>
       <c r="I37" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J37" t="inlineStr" s="5">
@@ -2411,12 +2440,12 @@
       </c>
       <c r="H38" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: API PUT /api/meetings/1 trả về HTTP 200 OK, cập nhật thành công các trường thông tin trong bảng Meetings và Bookings.</t>
         </is>
       </c>
       <c r="I38" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J38" t="inlineStr" s="5">
@@ -2472,12 +2501,12 @@
       </c>
       <c r="H39" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: API trả về đúng HTTP 404 Not Found kèm thông báo 'Cuộc họp với ID không tồn tại'.</t>
         </is>
       </c>
       <c r="I39" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J39" t="inlineStr" s="5">
@@ -2532,12 +2561,12 @@
       </c>
       <c r="H40" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: API trả về đúng HTTP 400 Bad Request kèm thông báo 'Vui lòng nhập đủ các trường bắt buộc'.</t>
         </is>
       </c>
       <c r="I40" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J40" t="inlineStr" s="5">
@@ -2592,12 +2621,12 @@
       </c>
       <c r="H41" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Hệ thống phát hiện dữ liệu không hợp lệ chính xác, hiển thị thông báo cảnh báo tương ứng và chặn gửi dữ liệu thành công.</t>
         </is>
       </c>
       <c r="I41" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J41" t="inlineStr" s="5">
@@ -2652,12 +2681,12 @@
       </c>
       <c r="H42" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: API trả về đúng HTTP 400 Bad Request kèm thông báo 'Thời gian kết thúc phải sau thời gian bắt đầu'.</t>
         </is>
       </c>
       <c r="I42" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J42" t="inlineStr" s="5">
@@ -2712,12 +2741,12 @@
       </c>
       <c r="H43" t="inlineStr" s="5">
         <is>
-          <t/>
+          <t>Đạt: Prepared Statement ngăn chặn triệt để SQL Injection, hệ thống an toàn và xử lý chuẩn xác.</t>
         </is>
       </c>
       <c r="I43" t="inlineStr" s="9">
         <is>
-          <t/>
+          <t>Pass</t>
         </is>
       </c>
       <c r="J43" t="inlineStr" s="5">

</xml_diff>